<commit_message>
Release v1.0.2: Add LATEST VERSION column to shotlist template
</commit_message>
<xml_diff>
--- a/resources/SHOTLIST_TEMPLATE.xlsx
+++ b/resources/SHOTLIST_TEMPLATE.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>PROJECT NAME</t>
   </si>
@@ -29,6 +29,9 @@
   </si>
   <si>
     <t>TIMECODE IN</t>
+  </si>
+  <si>
+    <t>LATEST VERSION</t>
   </si>
   <si>
     <t>DESCRIPTION</t>
@@ -103,12 +106,12 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -128,6 +131,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -352,9 +358,10 @@
     <col customWidth="1" min="1" max="1" width="27.75"/>
     <col customWidth="1" min="2" max="2" width="15.88"/>
     <col customWidth="1" min="3" max="3" width="14.13"/>
-    <col customWidth="1" min="4" max="4" width="31.5"/>
-    <col customWidth="1" min="5" max="5" width="16.75"/>
-    <col customWidth="1" min="6" max="6" width="27.5"/>
+    <col customWidth="1" min="4" max="4" width="23.63"/>
+    <col customWidth="1" min="5" max="5" width="31.5"/>
+    <col customWidth="1" min="6" max="6" width="16.75"/>
+    <col customWidth="1" min="7" max="7" width="27.5"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1">
@@ -370,6 +377,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" ht="63.75" customHeight="1">
       <c r="B2" s="4"/>
@@ -377,6 +385,7 @@
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
@@ -396,6 +405,9 @@
       </c>
       <c r="F3" s="6" t="s">
         <v>8</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -403,8 +415,9 @@
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
       <c r="D4" s="9"/>
-      <c r="E4" s="8"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Release v1.0.4: Added column Latest Version to Export
</commit_message>
<xml_diff>
--- a/resources/SHOTLIST_TEMPLATE.xlsx
+++ b/resources/SHOTLIST_TEMPLATE.xlsx
@@ -95,18 +95,32 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border/>
     <border>
       <top style="thick">
         <color rgb="FF000000"/>
       </top>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -137,6 +151,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -417,7 +434,7 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
       <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
+      <c r="G4" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>